<commit_message>
split det v stoch models
</commit_message>
<xml_diff>
--- a/DATA/production_capacity_scenarios/cap_builder.xlsx
+++ b/DATA/production_capacity_scenarios/cap_builder.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/DATA/production_capacity_scenarios/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uark-my.sharepoint.com/personal/uhorchak_uark_edu/Documents/Desktop/Vaccine_Tender/DATA/production_capacity_scenarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="278" documentId="8_{CA986233-5C84-4EAA-B96B-661799E682FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDF4F9CE-542A-4F7A-9DCD-734FC4397F51}"/>
+  <xr:revisionPtr revIDLastSave="284" documentId="8_{CA986233-5C84-4EAA-B96B-661799E682FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F093489-6990-4AB0-8A55-24CDB159A350}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CCA420AF-4493-4C79-A19E-AC0C61F28524}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{CCA420AF-4493-4C79-A19E-AC0C61F28524}"/>
   </bookViews>
   <sheets>
     <sheet name="starting_cap" sheetId="1" r:id="rId1"/>
@@ -698,10 +698,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1022,13 +1018,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAA7A5DA-6C9D-46FC-975A-A9F5DD878FF9}">
   <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1036,7 +1032,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1044,7 +1040,7 @@
         <v>977251.31527214276</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1052,7 +1048,7 @@
         <v>13328055.520714156</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1060,7 +1056,7 @@
         <v>321326687.20403224</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1068,7 +1064,7 @@
         <v>6402511.719496578</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -1076,7 +1072,7 @@
         <v>59151603.417757481</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -1084,7 +1080,7 @@
         <v>277874999.07853091</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -1092,7 +1088,7 @@
         <v>302888.81815348461</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -1100,7 +1096,7 @@
         <v>6311801.7126107905</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -1108,7 +1104,7 @@
         <v>66709612.957940787</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1116,7 +1112,7 @@
         <v>136545787.17132425</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1124,7 +1120,7 @@
         <v>266622339.29579192</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -1132,15 +1128,15 @@
         <v>3172885.866301666</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>31</v>
       </c>
       <c r="B14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>438402962.04456699</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -1148,7 +1144,7 @@
         <v>35984585.712862946</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -1156,7 +1152,7 @@
         <v>217521514.44316691</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -1172,30 +1168,30 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5B0376C-AE0A-41BC-8998-FF6C9C8BC443}">
   <dimension ref="A1:J49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -1221,7 +1217,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1236,18 +1232,18 @@
         <v>6402511.719496578</v>
       </c>
       <c r="E2">
-        <f t="shared" ref="E2:E49" si="0">D2*B2</f>
+        <f>D2*B2</f>
         <v>3958786.3845079578</v>
       </c>
       <c r="I2" t="s">
         <v>18</v>
       </c>
       <c r="J2">
-        <f t="shared" ref="J2:J16" si="1">SUMIF(A:A, I2, E:E)</f>
+        <f t="shared" ref="J2:J16" si="0">SUMIF(A:A, I2, E:E)</f>
         <v>12102355.415715292</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -1262,18 +1258,18 @@
         <v>6402511.719496578</v>
       </c>
       <c r="E3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E2:E49" si="1">D3*B3</f>
         <v>2443725.3349886201</v>
       </c>
       <c r="I3" t="s">
         <v>19</v>
       </c>
       <c r="J3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>55762252.537822999</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1288,18 +1284,18 @@
         <v>59151603.417757481</v>
       </c>
       <c r="E4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>46967196.599250063</v>
       </c>
       <c r="I4" t="s">
         <v>20</v>
       </c>
       <c r="J4">
-        <f t="shared" si="1"/>
-        <v>5457031.9499387406</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>77986389.151167125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -1314,18 +1310,18 @@
         <v>59151603.417757481</v>
       </c>
       <c r="E5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12184406.818507425</v>
       </c>
       <c r="I5" t="s">
         <v>21</v>
       </c>
       <c r="J5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>18909478.051597763</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -1340,18 +1336,18 @@
         <v>6311801.7126107905</v>
       </c>
       <c r="E6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6311801.7126107905</v>
       </c>
       <c r="I6" t="s">
         <v>22</v>
       </c>
       <c r="J6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>176656204.10945982</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1366,18 +1362,18 @@
         <v>66709612.957940787</v>
       </c>
       <c r="E7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>35030933.557310052</v>
       </c>
       <c r="I7" t="s">
         <v>16</v>
       </c>
       <c r="J7">
-        <f t="shared" si="1"/>
-        <v>1317354.7756154076</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>14503588.18448288</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1392,18 +1388,18 @@
         <v>66709612.957940787</v>
       </c>
       <c r="E8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>31678679.400630668</v>
       </c>
       <c r="I8" t="s">
         <v>23</v>
       </c>
       <c r="J8">
-        <f t="shared" si="1"/>
-        <v>379834532.08035249</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>414824585.3056196</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1418,18 +1414,18 @@
         <v>302888.81815348461</v>
       </c>
       <c r="E9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>302888.81815348461</v>
       </c>
       <c r="I9" t="s">
         <v>24</v>
       </c>
       <c r="J9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>102061729.61303598</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1444,18 +1440,18 @@
         <v>35984585.712862946</v>
       </c>
       <c r="E10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>31938848.527961027</v>
       </c>
       <c r="I10" t="s">
         <v>25</v>
       </c>
       <c r="J10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>89157748.448498234</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1470,18 +1466,18 @@
         <v>35984585.712862946</v>
       </c>
       <c r="E11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2728382.4092865069</v>
       </c>
       <c r="I11" t="s">
         <v>26</v>
       </c>
       <c r="J11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>31938848.527961027</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1496,18 +1492,18 @@
         <v>35984585.712862946</v>
       </c>
       <c r="E12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1317354.7756154076</v>
       </c>
       <c r="I12" t="s">
         <v>27</v>
       </c>
       <c r="J12">
-        <f t="shared" si="1"/>
-        <v>14015815.917442642</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>15219754.312615251</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -1522,18 +1518,18 @@
         <v>136545787.17132425</v>
       </c>
       <c r="E13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>101436558.60119651</v>
       </c>
       <c r="I13" t="s">
         <v>12</v>
       </c>
       <c r="J13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>127439682.10564198</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1548,18 +1544,18 @@
         <v>136545787.17132425</v>
       </c>
       <c r="E14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18909478.051597763</v>
       </c>
       <c r="I14" t="s">
         <v>28</v>
       </c>
       <c r="J14">
-        <f t="shared" si="1"/>
-        <v>42815576.129015923</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>56000384.381950192</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -1574,18 +1570,18 @@
         <v>136545787.17132425</v>
       </c>
       <c r="E15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4097395.1028146716</v>
       </c>
       <c r="I15" t="s">
         <v>15</v>
       </c>
       <c r="J15">
-        <f t="shared" si="1"/>
-        <v>101739447.41935</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>130015283.84818706</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -1600,18 +1596,18 @@
         <v>136545787.17132425</v>
       </c>
       <c r="E16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12102355.415715292</v>
       </c>
       <c r="I16" t="s">
         <v>29</v>
       </c>
       <c r="J16">
-        <f t="shared" si="1"/>
-        <v>581266772.68311989</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>754237778.20234299</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1626,11 +1622,11 @@
         <v>977251.31527214276</v>
       </c>
       <c r="E17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>828063.30500688718</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -1645,11 +1641,11 @@
         <v>977251.31527214276</v>
       </c>
       <c r="E18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>149188.01026525456</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -1664,11 +1660,11 @@
         <v>321326687.20403224</v>
       </c>
       <c r="E19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>235424959.37692702</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -1683,11 +1679,11 @@
         <v>321326687.20403224</v>
       </c>
       <c r="E20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>85901727.827104896</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>29</v>
       </c>
@@ -1702,11 +1698,11 @@
         <v>13328055.520714156</v>
       </c>
       <c r="E21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>11211272.916422246</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1721,11 +1717,11 @@
         <v>13328055.520714156</v>
       </c>
       <c r="E22">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2116782.6042918968</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -1737,14 +1733,14 @@
       </c>
       <c r="D23">
         <f>VLOOKUP(C23,starting_cap!$A$2:$B$17,2,FALSE)</f>
-        <v>0</v>
+        <v>438402962.04456699</v>
       </c>
       <c r="E23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>172971005.51922327</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -1756,14 +1752,14 @@
       </c>
       <c r="D24">
         <f>VLOOKUP(C24,starting_cap!$A$2:$B$17,2,FALSE)</f>
-        <v>0</v>
+        <v>438402962.04456699</v>
       </c>
       <c r="E24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>102061729.61303598</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>20</v>
       </c>
@@ -1775,14 +1771,14 @@
       </c>
       <c r="D25">
         <f>VLOOKUP(C25,starting_cap!$A$2:$B$17,2,FALSE)</f>
-        <v>0</v>
+        <v>438402962.04456699</v>
       </c>
       <c r="E25">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>72529357.20122838</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -1794,14 +1790,14 @@
       </c>
       <c r="D26">
         <f>VLOOKUP(C26,starting_cap!$A$2:$B$17,2,FALSE)</f>
-        <v>0</v>
+        <v>438402962.04456699</v>
       </c>
       <c r="E26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>34990053.22526715</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -1813,14 +1809,14 @@
       </c>
       <c r="D27">
         <f>VLOOKUP(C27,starting_cap!$A$2:$B$17,2,FALSE)</f>
-        <v>0</v>
+        <v>438402962.04456699</v>
       </c>
       <c r="E27">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>28275836.428837061</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>16</v>
       </c>
@@ -1832,14 +1828,14 @@
       </c>
       <c r="D28">
         <f>VLOOKUP(C28,starting_cap!$A$2:$B$17,2,FALSE)</f>
-        <v>0</v>
+        <v>438402962.04456699</v>
       </c>
       <c r="E28">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>13186233.408867473</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -1851,14 +1847,14 @@
       </c>
       <c r="D29">
         <f>VLOOKUP(C29,starting_cap!$A$2:$B$17,2,FALSE)</f>
-        <v>0</v>
+        <v>438402962.04456699</v>
       </c>
       <c r="E29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>13184808.252934271</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>27</v>
       </c>
@@ -1870,14 +1866,14 @@
       </c>
       <c r="D30">
         <f>VLOOKUP(C30,starting_cap!$A$2:$B$17,2,FALSE)</f>
-        <v>0</v>
+        <v>438402962.04456699</v>
       </c>
       <c r="E30">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="1"/>
+        <v>1203938.3951726083</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -1892,11 +1888,11 @@
         <v>226180575.91757733</v>
       </c>
       <c r="E31">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>127439682.10564198</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -1911,11 +1907,11 @@
         <v>226180575.91757733</v>
       </c>
       <c r="E32">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>92167337.98075521</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>29</v>
       </c>
@@ -1930,11 +1926,11 @@
         <v>226180575.91757733</v>
       </c>
       <c r="E33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6573555.8311797418</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>29</v>
       </c>
@@ -1949,11 +1945,11 @@
         <v>277874999.07853091</v>
       </c>
       <c r="E34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>140349220.87761426</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>22</v>
       </c>
@@ -1968,11 +1964,11 @@
         <v>277874999.07853091</v>
       </c>
       <c r="E35">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>66588024.007865503</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>25</v>
       </c>
@@ -1987,11 +1983,11 @@
         <v>277874999.07853091</v>
       </c>
       <c r="E36">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>53381673.945052892</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>27</v>
       </c>
@@ -2006,11 +2002,11 @@
         <v>277874999.07853091</v>
       </c>
       <c r="E37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>14015815.917442642</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>28</v>
       </c>
@@ -2025,11 +2021,11 @@
         <v>277874999.07853091</v>
       </c>
       <c r="E38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3540264.3305556043</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>23</v>
       </c>
@@ -2044,11 +2040,11 @@
         <v>217521514.44316691</v>
       </c>
       <c r="E39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>199037083.86320585</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>29</v>
       </c>
@@ -2063,11 +2059,11 @@
         <v>217521514.44316691</v>
       </c>
       <c r="E40">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>13027398.630022222</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>20</v>
       </c>
@@ -2082,11 +2078,11 @@
         <v>217521514.44316691</v>
       </c>
       <c r="E41">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5457031.9499387406</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -2101,11 +2097,11 @@
         <v>266622339.29579192</v>
       </c>
       <c r="E42">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>93894420.830715775</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>29</v>
       </c>
@@ -2120,11 +2116,11 @@
         <v>266622339.29579192</v>
       </c>
       <c r="E43">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>84982734.46390073</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -2139,11 +2135,11 @@
         <v>266622339.29579192</v>
       </c>
       <c r="E44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>51233055.894558154</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>28</v>
       </c>
@@ -2158,11 +2154,11 @@
         <v>266622339.29579192</v>
       </c>
       <c r="E45">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>36512128.106616735</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>22</v>
       </c>
@@ -2177,11 +2173,11 @@
         <v>3172885.866301666</v>
       </c>
       <c r="E46">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1872569.848079198</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>19</v>
       </c>
@@ -2196,11 +2192,11 @@
         <v>3172885.866301666</v>
       </c>
       <c r="E47">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>570410.25875688565</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>29</v>
       </c>
@@ -2215,11 +2211,11 @@
         <v>3172885.866301666</v>
       </c>
       <c r="E48">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>559635.41287587222</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>28</v>
       </c>
@@ -2234,7 +2230,7 @@
         <v>3172885.866301666</v>
       </c>
       <c r="E49">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>170270.34658970434</v>
       </c>
     </row>

</xml_diff>